<commit_message>
Feat:Adicionando o teste de impressão de ordens
</commit_message>
<xml_diff>
--- a/data/output/Cenários de Testes Unitários e Parciais - PM-Manutenção  1.xlsx
+++ b/data/output/Cenários de Testes Unitários e Parciais - PM-Manutenção  1.xlsx
@@ -194,7 +194,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="39">
+  <fills count="38">
     <fill>
       <patternFill/>
     </fill>
@@ -402,11 +402,6 @@
         <fgColor rgb="00E2F0D9"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="13">
     <border>
@@ -608,7 +603,7 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="33" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -661,10 +656,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="38" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="38" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -1192,7 +1183,7 @@
       </c>
       <c r="H2" s="22" t="inlineStr">
         <is>
-          <t>Nota 11054898 gravada | POPUP: Parceiro || Informação objeto || Modif.prioridade</t>
+          <t>Nota 15411955 gravada | POPUP: Parceiro || Informação objeto || Modif.prioridade</t>
         </is>
       </c>
       <c r="I2" s="22" t="inlineStr"/>
@@ -1206,7 +1197,7 @@
       </c>
       <c r="L2" s="23" t="inlineStr">
         <is>
-          <t>\evidence\c87c64dfa9_Testes_unitários_r2_IW21_RUN_20260310_140826.png</t>
+          <t>\evidence\445129883a_Testes_unitários_r2_IW21_RUN_20260311_083732.png</t>
         </is>
       </c>
     </row>
@@ -1246,7 +1237,7 @@
       </c>
       <c r="H3" s="22" t="inlineStr">
         <is>
-          <t>Executado com sucesso | POPUP: Parceiro || Informação objeto || Informação || Informação</t>
+          <t>Ordem 103548367 com nota 15411956 gravada | POPUP: Parceiro || Informação objeto || Modif.prioridade</t>
         </is>
       </c>
       <c r="I3" s="22" t="inlineStr"/>
@@ -1260,7 +1251,7 @@
       </c>
       <c r="L3" s="23" t="inlineStr">
         <is>
-          <t>\evidence\c87c64dfa9_Testes_unitários_r3_IW31_RUN_20260310_140843.png</t>
+          <t>\evidence\445129883a_Testes_unitários_r3_IW31_RUN_20260311_083758.png</t>
         </is>
       </c>
     </row>
@@ -1300,7 +1291,7 @@
       </c>
       <c r="H4" s="22" t="inlineStr">
         <is>
-          <t>Executado com sucesso | POPUP: Parceiro || Informação objeto || Informação || Informação</t>
+          <t>Ordem 140529256 com nota 15411957 gravada | POPUP: Parceiro || Informação objeto || Modif.prioridade</t>
         </is>
       </c>
       <c r="I4" s="22" t="inlineStr"/>
@@ -1314,7 +1305,7 @@
       </c>
       <c r="L4" s="23" t="inlineStr">
         <is>
-          <t>\evidence\c87c64dfa9_Testes_unitários_r4_IW31_RUN_20260310_140901.png</t>
+          <t>\evidence\445129883a_Testes_unitários_r4_IW31_RUN_20260311_083824.png</t>
         </is>
       </c>
     </row>
@@ -1342,37 +1333,33 @@
           <t>Equipamento: 10141343 | Texto Breve: teste | TipoAtvMnt: 19 | Prioridade: 3  | Trabalho: 1 | Nº Colaboradores: 1</t>
         </is>
       </c>
-      <c r="F5" s="27" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="F5" s="21" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G5" s="20" t="inlineStr">
         <is>
-          <t>STATUSBAR</t>
-        </is>
-      </c>
-      <c r="H5" s="28" t="inlineStr">
-        <is>
-          <t>Erro não identificado</t>
-        </is>
-      </c>
-      <c r="I5" s="28" t="inlineStr">
-        <is>
-          <t>Verificar mensagem SAP e evidência.</t>
-        </is>
-      </c>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H5" s="22" t="inlineStr">
+        <is>
+          <t>Ordem 121105181 com nota 15411958 gravada | POPUP: Parceiro || Informação objeto || Modif.prioridade</t>
+        </is>
+      </c>
+      <c r="I5" s="22" t="inlineStr"/>
       <c r="J5" s="20" t="n">
-        <v>65</v>
+        <v>100</v>
       </c>
       <c r="K5" s="22" t="inlineStr">
         <is>
-          <t>Primeira ocorrência deste erro. Análise baseada na mensagem SAP e no dump.</t>
+          <t>Execução concluída sem erros.</t>
         </is>
       </c>
       <c r="L5" s="23" t="inlineStr">
         <is>
-          <t>\evidence\c87c64dfa9_Testes_unitários_r5_IW31_RUN_20260310_140919.png</t>
+          <t>\evidence\445129883a_Testes_unitários_r5_IW31_RUN_20260311_083849.png</t>
         </is>
       </c>
     </row>
@@ -1408,7 +1395,7 @@
       </c>
       <c r="H6" s="22" t="inlineStr">
         <is>
-          <t>Executado com sucesso</t>
+          <t>Fluxo IW32 de impressão executado com sucesso</t>
         </is>
       </c>
       <c r="I6" s="22" t="inlineStr"/>
@@ -1422,7 +1409,7 @@
       </c>
       <c r="L6" s="23" t="inlineStr">
         <is>
-          <t>\evidence\c87c64dfa9_Testes_unitários_r6_IW32_RUN_20260310_140923.png</t>
+          <t>\evidence\445129883a_Testes_unitários_r6_IW32_RUN_20260311_083906.png</t>
         </is>
       </c>
     </row>
@@ -1487,7 +1474,7 @@
       <c r="B11" s="20" t="n"/>
       <c r="C11" s="20" t="n"/>
       <c r="D11" s="20" t="n"/>
-      <c r="E11" s="29" t="n"/>
+      <c r="E11" s="27" t="n"/>
       <c r="F11" s="20" t="n"/>
       <c r="G11" s="20" t="n"/>
       <c r="H11" s="20" t="n"/>

</xml_diff>